<commit_message>
[Data] uint -> int 타입 변경
</commit_message>
<xml_diff>
--- a/Assets/06 Data/ExcelData/dt_ammo_item.xlsx
+++ b/Assets/06 Data/ExcelData/dt_ammo_item.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Genie\Desktop\duckov-clone\Assets\06 Data\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4812C49B-97E3-4CFB-BBDD-E18BAC112679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2C75CB-3C81-4CA6-B697-459A2B4F57CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11295" xr2:uid="{3E9BE2B3-753F-4CB8-8C74-169030718F3F}"/>
+    <workbookView xWindow="6750" yWindow="2775" windowWidth="20595" windowHeight="11295" xr2:uid="{3E9BE2B3-753F-4CB8-8C74-169030718F3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -66,10 +66,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>uint</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>string</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -143,6 +139,10 @@
   </si>
   <si>
     <t>MaxStackSize</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -606,13 +606,13 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>4</v>
@@ -624,68 +624,68 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="I2" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>9</v>
-      </c>
       <c r="H3" s="4" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -693,13 +693,13 @@
         <v>595</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>0</v>
@@ -722,13 +722,13 @@
         <v>622</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>1</v>

</xml_diff>